<commit_message>
fix: correct catering template formula (I17→I23) + regenerate all Excel files
The Presupuesto sheet in 06-catering referenced an empty row (I17) instead
of the actual COSTE TOTAL DEL PLATO cell (I23), causing #VALUE! cascade
errors. Fixed the reference and regenerated all 12 templates from script.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/dl/ke-17b9.xlsx
+++ b/public/dl/ke-17b9.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView activeTab="0" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tostada Aguacate" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Açaí Bowl" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eggs Benedict" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Tostada Aguacate" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Açaí Bowl" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Eggs Benedict" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Tostada Aguacate'!$A$1:$I$26</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'Açaí Bowl'!$A$1:$I$26</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">'Eggs Benedict'!$A$1:$I$25</definedName>
+    <definedName localSheetId="1" name="_xlnm.Print_Area">'Tostada Aguacate'!$A$1:$I$26</definedName>
+    <definedName localSheetId="2" name="_xlnm.Print_Area">'Açaí Bowl'!$A$1:$I$26</definedName>
+    <definedName localSheetId="3" name="_xlnm.Print_Area">'Eggs Benedict'!$A$1:$I$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -24,9 +24,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="#,##0.00 €"/>
-    <numFmt numFmtId="165" formatCode="0.000"/>
-    <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt formatCode="#,##0.00 €" numFmtId="164"/>
+    <numFmt formatCode="0.000" numFmtId="165"/>
+    <numFmt formatCode="0.0%" numFmtId="166"/>
   </numFmts>
   <fonts count="18">
     <font>
@@ -353,110 +353,110 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
   </cellStyleXfs>
   <cellXfs count="48">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="6" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="11" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="1" fillId="0" fontId="8" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf borderId="1" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="14" fillId="3" fontId="12" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf borderId="2" fillId="2" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="3" fillId="2" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="14" fillId="4" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="14" fillId="4" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="14" fillId="4" fontId="5" numFmtId="164" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="14" fillId="4" fontId="5" numFmtId="165" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="5" fillId="4" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="14" fillId="4" fontId="5" numFmtId="9" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="14" fillId="0" fontId="13" numFmtId="165" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="14" fillId="0" fontId="13" numFmtId="164" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf borderId="4" fillId="2" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="5" fillId="2" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="0" fillId="4" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf borderId="10" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="12" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="13" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="14" fillId="4" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="14" fillId="4" fontId="0" numFmtId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="14" fillId="0" fontId="0" numFmtId="165" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="14" fillId="0" fontId="0" numFmtId="164" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="6" fillId="2" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="7" fillId="2" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="14" fillId="5" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf borderId="14" fillId="5" fontId="4" numFmtId="164" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="14" fillId="0" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf borderId="14" fillId="0" fontId="13" numFmtId="164" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="14" fillId="6" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="6" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf borderId="14" fillId="6" fontId="15" numFmtId="164" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="14" fillId="0" fontId="13" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="16" fillId="4" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="14" fillId="4" fontId="16" numFmtId="9" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="14" fillId="0" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf borderId="14" fillId="0" fontId="4" numFmtId="164" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="14" fillId="6" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="6" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="13" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="14" fillId="6" fontId="17" numFmtId="164" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="14" fillId="0" fontId="13" numFmtId="166" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle builtinId="0" hidden="0" name="Normal" xfId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium9"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -821,8 +821,8 @@
   <dimension ref="B2:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="80" customWidth="1" min="2" max="2"/>
+    <col customWidth="1" max="1" min="1" width="3"/>
+    <col customWidth="1" max="2" min="2" width="80"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -898,7 +898,7 @@
   <mergeCells count="1">
     <mergeCell ref="B2"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>
 </file>
 
@@ -912,18 +912,18 @@
   <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="3" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
+    <col customWidth="1" max="1" min="1" width="25"/>
+    <col customWidth="1" max="2" min="2" width="16"/>
+    <col customWidth="1" max="3" min="3" width="12"/>
+    <col customWidth="1" max="4" min="4" width="14"/>
+    <col customWidth="1" max="5" min="5" width="12"/>
+    <col customWidth="1" max="6" min="6" width="12"/>
+    <col customWidth="1" max="7" min="7" width="10"/>
+    <col customWidth="1" max="8" min="8" width="14"/>
+    <col customWidth="1" max="9" min="9" width="14"/>
+    <col customWidth="1" max="10" min="10" width="3"/>
+    <col customWidth="1" max="11" min="11" width="20"/>
+    <col customWidth="1" max="12" min="12" width="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1479,30 +1479,30 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="K15:L15"/>
     <mergeCell ref="A18:H18"/>
+    <mergeCell ref="K8:L9"/>
+    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A20:H20"/>
     <mergeCell ref="A26:H26"/>
-    <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A25:H25"/>
-    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A1:I1"/>
     <mergeCell ref="A24:H24"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="A19:G19"/>
+    <mergeCell ref="A23:H23"/>
     <mergeCell ref="A22:G22"/>
-    <mergeCell ref="K15:L15"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A23:H23"/>
-    <mergeCell ref="A19:G19"/>
-    <mergeCell ref="K8:L9"/>
-    <mergeCell ref="K3:L3"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="B5 B6 B7 B8 B9 B10 B11 B12 B13 B14 B15 B16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Categoría inválida" error="Selecciona una categoría válida" type="list">
+    <dataValidation allowBlank="1" error="Selecciona una categoría válida" errorTitle="Categoría inválida" showDropDown="0" showErrorMessage="0" showInputMessage="0" sqref="B5 B6 B7 B8 B9 B10 B11 B12 B13 B14 B15 B16" type="list">
       <formula1>"Carne roja,Aves,Pescado,Marisco,Verdura hoja,Verdura raíz,Fruta,Lácteos,Secos/granos,Congelados,Pan/bollería,Huevos,Aceites/grasas,Especias/hierbas,Chocolate/cacao,Bebidas/licores"</formula1>
     </dataValidation>
-    <dataValidation sqref="C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation allowBlank="1" showDropDown="0" showErrorMessage="0" showInputMessage="0" sqref="C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16" type="list">
       <formula1>"kg,g,L,ml,cl,ud,docena,manojo,sobre,lata,botella"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
+  <pageSetup fitToHeight="0" fitToWidth="1" orientation="landscape"/>
 </worksheet>
 </file>
 
@@ -1516,18 +1516,18 @@
   <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="3" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
+    <col customWidth="1" max="1" min="1" width="25"/>
+    <col customWidth="1" max="2" min="2" width="16"/>
+    <col customWidth="1" max="3" min="3" width="12"/>
+    <col customWidth="1" max="4" min="4" width="14"/>
+    <col customWidth="1" max="5" min="5" width="12"/>
+    <col customWidth="1" max="6" min="6" width="12"/>
+    <col customWidth="1" max="7" min="7" width="10"/>
+    <col customWidth="1" max="8" min="8" width="14"/>
+    <col customWidth="1" max="9" min="9" width="14"/>
+    <col customWidth="1" max="10" min="10" width="3"/>
+    <col customWidth="1" max="11" min="11" width="20"/>
+    <col customWidth="1" max="12" min="12" width="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2083,30 +2083,30 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="K15:L15"/>
     <mergeCell ref="A18:H18"/>
+    <mergeCell ref="K8:L9"/>
+    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A20:H20"/>
     <mergeCell ref="A26:H26"/>
-    <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A25:H25"/>
-    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A1:I1"/>
     <mergeCell ref="A24:H24"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="A19:G19"/>
+    <mergeCell ref="A23:H23"/>
     <mergeCell ref="A22:G22"/>
-    <mergeCell ref="K15:L15"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A23:H23"/>
-    <mergeCell ref="A19:G19"/>
-    <mergeCell ref="K8:L9"/>
-    <mergeCell ref="K3:L3"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="B5 B6 B7 B8 B9 B10 B11 B12 B13 B14 B15 B16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Categoría inválida" error="Selecciona una categoría válida" type="list">
+    <dataValidation allowBlank="1" error="Selecciona una categoría válida" errorTitle="Categoría inválida" showDropDown="0" showErrorMessage="0" showInputMessage="0" sqref="B5 B6 B7 B8 B9 B10 B11 B12 B13 B14 B15 B16" type="list">
       <formula1>"Carne roja,Aves,Pescado,Marisco,Verdura hoja,Verdura raíz,Fruta,Lácteos,Secos/granos,Congelados,Pan/bollería,Huevos,Aceites/grasas,Especias/hierbas,Chocolate/cacao,Bebidas/licores"</formula1>
     </dataValidation>
-    <dataValidation sqref="C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation allowBlank="1" showDropDown="0" showErrorMessage="0" showInputMessage="0" sqref="C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16" type="list">
       <formula1>"kg,g,L,ml,cl,ud,docena,manojo,sobre,lata,botella"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
+  <pageSetup fitToHeight="0" fitToWidth="1" orientation="landscape"/>
 </worksheet>
 </file>
 
@@ -2120,18 +2120,18 @@
   <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="3" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
+    <col customWidth="1" max="1" min="1" width="25"/>
+    <col customWidth="1" max="2" min="2" width="16"/>
+    <col customWidth="1" max="3" min="3" width="12"/>
+    <col customWidth="1" max="4" min="4" width="14"/>
+    <col customWidth="1" max="5" min="5" width="12"/>
+    <col customWidth="1" max="6" min="6" width="12"/>
+    <col customWidth="1" max="7" min="7" width="10"/>
+    <col customWidth="1" max="8" min="8" width="14"/>
+    <col customWidth="1" max="9" min="9" width="14"/>
+    <col customWidth="1" max="10" min="10" width="3"/>
+    <col customWidth="1" max="11" min="11" width="20"/>
+    <col customWidth="1" max="12" min="12" width="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2648,29 +2648,29 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="K15:L15"/>
+    <mergeCell ref="K8:L9"/>
+    <mergeCell ref="A25:H25"/>
     <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A17:H17"/>
     <mergeCell ref="A18:G18"/>
-    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A22:H22"/>
+    <mergeCell ref="A19:H19"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A24:H24"/>
+    <mergeCell ref="K3:L3"/>
     <mergeCell ref="A21:G21"/>
-    <mergeCell ref="A24:H24"/>
-    <mergeCell ref="K15:L15"/>
-    <mergeCell ref="A22:H22"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A19:H19"/>
     <mergeCell ref="A23:H23"/>
-    <mergeCell ref="K8:L9"/>
-    <mergeCell ref="K3:L3"/>
-    <mergeCell ref="A17:H17"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="B5 B6 B7 B8 B9 B10 B11 B12 B13 B14 B15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Categoría inválida" error="Selecciona una categoría válida" type="list">
+    <dataValidation allowBlank="1" error="Selecciona una categoría válida" errorTitle="Categoría inválida" showDropDown="0" showErrorMessage="0" showInputMessage="0" sqref="B5 B6 B7 B8 B9 B10 B11 B12 B13 B14 B15" type="list">
       <formula1>"Carne roja,Aves,Pescado,Marisco,Verdura hoja,Verdura raíz,Fruta,Lácteos,Secos/granos,Congelados,Pan/bollería,Huevos,Aceites/grasas,Especias/hierbas,Chocolate/cacao,Bebidas/licores"</formula1>
     </dataValidation>
-    <dataValidation sqref="C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation allowBlank="1" showDropDown="0" showErrorMessage="0" showInputMessage="0" sqref="C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15" type="list">
       <formula1>"kg,g,L,ml,cl,ud,docena,manojo,sobre,lata,botella"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
+  <pageSetup fitToHeight="0" fitToWidth="1" orientation="landscape"/>
 </worksheet>
 </file>
</xml_diff>